<commit_message>
combined_probable_trained_model with 84.62% of accuracy
</commit_message>
<xml_diff>
--- a/data/Complete_dataset.xlsx
+++ b/data/Complete_dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alvar\Repository\Roman-Chebba-agriculture\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\OneDrive\Documents\repos\Roman-Chebba-agriculture\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF6732F3-8DFF-4066-A081-E92AE62B92A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CBA31E-138D-44D2-A923-F3859B266EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legend" sheetId="1" r:id="rId1"/>
@@ -18,19 +18,6 @@
     <sheet name="Other sites" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -1689,20 +1676,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="53.3984375" customWidth="1"/>
-    <col min="2" max="2" width="78.73046875" customWidth="1"/>
-    <col min="3" max="3" width="52.73046875" customWidth="1"/>
+    <col min="1" max="1" width="53.42578125" customWidth="1"/>
+    <col min="2" max="2" width="78.7109375" customWidth="1"/>
+    <col min="3" max="3" width="52.7109375" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="19.73046875" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="10" width="18" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="34.15" x14ac:dyDescent="1.05">
+    <row r="1" spans="1:11" ht="34.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="20" t="s">
         <v>205</v>
       </c>
@@ -1710,7 +1697,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1718,7 +1705,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1726,7 +1713,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>10</v>
       </c>
@@ -1734,7 +1721,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>181</v>
       </c>
@@ -1742,7 +1729,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>182</v>
       </c>
@@ -1750,7 +1737,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>13</v>
       </c>
@@ -1758,12 +1745,12 @@
         <v>187</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="68.25" x14ac:dyDescent="1.05">
+    <row r="10" spans="1:11" ht="69" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="18" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>123</v>
       </c>
@@ -1795,7 +1782,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>58</v>
       </c>
@@ -1827,7 +1814,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>68</v>
       </c>
@@ -1859,7 +1846,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -1891,7 +1878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -1923,7 +1910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -1943,7 +1930,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>66</v>
       </c>
@@ -1963,7 +1950,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -1983,7 +1970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -2003,7 +1990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>201</v>
       </c>
@@ -2017,7 +2004,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>202</v>
       </c>
@@ -2031,7 +2018,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>203</v>
       </c>
@@ -2045,12 +2032,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>162</v>
       </c>
@@ -2058,7 +2045,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>127</v>
       </c>
@@ -2066,7 +2053,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>128</v>
       </c>
@@ -2074,7 +2061,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>166</v>
       </c>
@@ -2082,7 +2069,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>168</v>
       </c>
@@ -2090,7 +2077,7 @@
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -2112,30 +2099,30 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AB93"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.3984375" style="16"/>
-    <col min="2" max="3" width="11.3984375" style="2"/>
-    <col min="4" max="6" width="43.73046875" customWidth="1"/>
-    <col min="7" max="7" width="35.1328125" customWidth="1"/>
-    <col min="8" max="9" width="11.3984375" style="15"/>
-    <col min="10" max="10" width="11.3984375" style="10"/>
-    <col min="13" max="13" width="11.3984375" style="11"/>
-    <col min="14" max="14" width="11.3984375" style="10"/>
-    <col min="16" max="16" width="14.86328125" customWidth="1"/>
-    <col min="17" max="17" width="11.3984375" style="11"/>
-    <col min="18" max="18" width="11.3984375" style="10"/>
+    <col min="1" max="1" width="11.42578125" style="16"/>
+    <col min="2" max="3" width="11.42578125" style="2"/>
+    <col min="4" max="6" width="43.7109375" customWidth="1"/>
+    <col min="7" max="7" width="35.140625" customWidth="1"/>
+    <col min="8" max="9" width="11.42578125" style="15"/>
+    <col min="10" max="10" width="11.42578125" style="10"/>
+    <col min="13" max="13" width="11.42578125" style="11"/>
+    <col min="14" max="14" width="11.42578125" style="10"/>
+    <col min="16" max="16" width="14.85546875" customWidth="1"/>
+    <col min="17" max="17" width="11.42578125" style="11"/>
+    <col min="18" max="18" width="11.42578125" style="10"/>
     <col min="20" max="20" width="18" customWidth="1"/>
-    <col min="21" max="21" width="20.265625" customWidth="1"/>
-    <col min="22" max="22" width="41.265625" customWidth="1"/>
+    <col min="21" max="21" width="20.28515625" customWidth="1"/>
+    <col min="22" max="22" width="41.28515625" customWidth="1"/>
     <col min="23" max="23" width="38" customWidth="1"/>
-    <col min="24" max="24" width="11.3984375" style="11"/>
-    <col min="25" max="25" width="18.1328125" style="10" customWidth="1"/>
+    <col min="24" max="24" width="11.42578125" style="11"/>
+    <col min="25" max="25" width="18.140625" style="10" customWidth="1"/>
     <col min="26" max="26" width="19" customWidth="1"/>
-    <col min="27" max="27" width="25.59765625" style="11" customWidth="1"/>
+    <col min="27" max="27" width="25.5703125" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:28" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="33" t="s">
         <v>206</v>
       </c>
@@ -2221,7 +2208,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
         <v>321</v>
       </c>
@@ -2304,7 +2291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
         <v>264</v>
       </c>
@@ -2385,7 +2372,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>266</v>
       </c>
@@ -2469,7 +2456,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>343</v>
       </c>
@@ -2553,7 +2540,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>267</v>
       </c>
@@ -2636,7 +2623,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>295</v>
       </c>
@@ -2717,7 +2704,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>320</v>
       </c>
@@ -2800,7 +2787,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>318</v>
       </c>
@@ -2881,7 +2868,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
         <v>297</v>
       </c>
@@ -2964,7 +2951,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
         <v>316</v>
       </c>
@@ -3045,7 +3032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
         <v>273</v>
       </c>
@@ -3128,7 +3115,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
         <v>271</v>
       </c>
@@ -3209,7 +3196,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>260</v>
       </c>
@@ -3292,7 +3279,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
         <v>259</v>
       </c>
@@ -3375,7 +3362,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
         <v>261</v>
       </c>
@@ -3458,7 +3445,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
         <v>262</v>
       </c>
@@ -3539,7 +3526,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
         <v>269</v>
       </c>
@@ -3623,7 +3610,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
         <v>275</v>
       </c>
@@ -3703,7 +3690,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
         <v>277</v>
       </c>
@@ -3783,7 +3770,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
         <v>285</v>
       </c>
@@ -3867,7 +3854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
         <v>287</v>
       </c>
@@ -3951,7 +3938,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>289</v>
       </c>
@@ -4032,7 +4019,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
         <v>283</v>
       </c>
@@ -4113,7 +4100,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
         <v>281</v>
       </c>
@@ -4194,7 +4181,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
         <v>279</v>
       </c>
@@ -4276,7 +4263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
         <v>256</v>
       </c>
@@ -4358,7 +4345,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
         <v>258</v>
       </c>
@@ -4440,7 +4427,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="26" t="s">
         <v>254</v>
       </c>
@@ -4526,7 +4513,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
         <v>314</v>
       </c>
@@ -4609,7 +4596,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
         <v>253</v>
       </c>
@@ -4623,7 +4610,7 @@
         <v>72</v>
       </c>
       <c r="E31" s="27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31" s="27"/>
       <c r="G31" s="16" t="s">
@@ -4690,7 +4677,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
         <v>250</v>
       </c>
@@ -4771,7 +4758,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" s="26" t="s">
         <v>248</v>
       </c>
@@ -4854,7 +4841,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
         <v>252</v>
       </c>
@@ -4935,7 +4922,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" s="26" t="s">
         <v>246</v>
       </c>
@@ -5018,7 +5005,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" s="26" t="s">
         <v>245</v>
       </c>
@@ -5101,7 +5088,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" s="26" t="s">
         <v>244</v>
       </c>
@@ -5184,7 +5171,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" s="26" t="s">
         <v>242</v>
       </c>
@@ -5269,7 +5256,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A39" s="26" t="s">
         <v>349</v>
       </c>
@@ -5356,7 +5343,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A40" s="26" t="s">
         <v>240</v>
       </c>
@@ -5437,7 +5424,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A41" s="26" t="s">
         <v>239</v>
       </c>
@@ -5520,7 +5507,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A42" s="26" t="s">
         <v>212</v>
       </c>
@@ -5604,7 +5591,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A43" s="26" t="s">
         <v>213</v>
       </c>
@@ -5687,7 +5674,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A44" s="26" t="s">
         <v>210</v>
       </c>
@@ -5770,7 +5757,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A45" s="26" t="s">
         <v>209</v>
       </c>
@@ -5853,7 +5840,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A46" s="26" t="s">
         <v>208</v>
       </c>
@@ -5936,7 +5923,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A47" s="26" t="s">
         <v>207</v>
       </c>
@@ -6019,7 +6006,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A48" s="26" t="s">
         <v>215</v>
       </c>
@@ -6104,7 +6091,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A49" s="26" t="s">
         <v>214</v>
       </c>
@@ -6187,7 +6174,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A50" s="26" t="s">
         <v>238</v>
       </c>
@@ -6270,7 +6257,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A51" s="26" t="s">
         <v>236</v>
       </c>
@@ -6353,7 +6340,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A52" s="26" t="s">
         <v>235</v>
       </c>
@@ -6440,7 +6427,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A53" s="26" t="s">
         <v>352</v>
       </c>
@@ -6527,7 +6514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A54" s="26" t="s">
         <v>234</v>
       </c>
@@ -6612,7 +6599,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A55" s="26" t="s">
         <v>231</v>
       </c>
@@ -6699,7 +6686,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A56" s="26" t="s">
         <v>232</v>
       </c>
@@ -6782,7 +6769,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A57" s="26" t="s">
         <v>233</v>
       </c>
@@ -6865,7 +6852,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A58" s="26" t="s">
         <v>225</v>
       </c>
@@ -6946,7 +6933,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A59" s="26" t="s">
         <v>227</v>
       </c>
@@ -7033,7 +7020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A60" s="26" t="s">
         <v>312</v>
       </c>
@@ -7046,10 +7033,10 @@
       <c r="D60" s="25" t="s">
         <v>313</v>
       </c>
-      <c r="E60" s="25"/>
-      <c r="F60" s="25">
+      <c r="E60" s="25">
         <v>1</v>
       </c>
+      <c r="F60" s="25"/>
       <c r="G60" t="s">
         <v>345</v>
       </c>
@@ -7118,7 +7105,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A61" s="26" t="s">
         <v>291</v>
       </c>
@@ -7199,7 +7186,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A62" s="26" t="s">
         <v>292</v>
       </c>
@@ -7282,7 +7269,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A63" s="26" t="s">
         <v>306</v>
       </c>
@@ -7365,7 +7352,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A64" s="26" t="s">
         <v>304</v>
       </c>
@@ -7448,7 +7435,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A65" s="26" t="s">
         <v>308</v>
       </c>
@@ -7532,7 +7519,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A66" s="26" t="s">
         <v>325</v>
       </c>
@@ -7613,7 +7600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A67" s="26" t="s">
         <v>305</v>
       </c>
@@ -7696,7 +7683,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A68" s="26" t="s">
         <v>302</v>
       </c>
@@ -7779,7 +7766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A69" s="26" t="s">
         <v>300</v>
       </c>
@@ -7862,7 +7849,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A70" s="26" t="s">
         <v>299</v>
       </c>
@@ -7949,7 +7936,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A71" s="26" t="s">
         <v>303</v>
       </c>
@@ -8032,7 +8019,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A72" s="26" t="s">
         <v>324</v>
       </c>
@@ -8117,7 +8104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A73" s="26" t="s">
         <v>322</v>
       </c>
@@ -8204,7 +8191,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A74" s="26" t="s">
         <v>329</v>
       </c>
@@ -8287,7 +8274,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A75" s="26" t="s">
         <v>333</v>
       </c>
@@ -8370,7 +8357,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A76" s="26" t="s">
         <v>331</v>
       </c>
@@ -8457,7 +8444,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A77" s="26" t="s">
         <v>327</v>
       </c>
@@ -8538,7 +8525,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A78" s="16" t="s">
         <v>335</v>
       </c>
@@ -8625,7 +8612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A79" s="16" t="s">
         <v>337</v>
       </c>
@@ -8706,7 +8693,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
         <v>339</v>
       </c>
@@ -8787,7 +8774,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A81" s="16" t="s">
         <v>223</v>
       </c>
@@ -8868,7 +8855,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A82" s="16" t="s">
         <v>357</v>
       </c>
@@ -8949,7 +8936,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A83" s="16" t="s">
         <v>222</v>
       </c>
@@ -9034,7 +9021,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A84" s="16" t="s">
         <v>311</v>
       </c>
@@ -9115,7 +9102,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A85" s="16" t="s">
         <v>219</v>
       </c>
@@ -9196,7 +9183,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A86" s="16" t="s">
         <v>221</v>
       </c>
@@ -9279,7 +9266,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A87" s="16" t="s">
         <v>218</v>
       </c>
@@ -9366,7 +9353,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A88" s="16" t="s">
         <v>228</v>
       </c>
@@ -9449,7 +9436,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A89" s="16" t="s">
         <v>229</v>
       </c>
@@ -9532,7 +9519,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A90" s="16" t="s">
         <v>230</v>
       </c>
@@ -9615,7 +9602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="91" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A91" s="16" t="s">
         <v>310</v>
       </c>
@@ -9698,7 +9685,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A92" s="16" t="s">
         <v>367</v>
       </c>
@@ -9781,7 +9768,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A93" s="16" t="s">
         <v>216</v>
       </c>
@@ -9874,27 +9861,27 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AE53"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="34.1328125" customWidth="1"/>
-    <col min="4" max="4" width="16.265625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.86328125" style="2" customWidth="1"/>
-    <col min="9" max="14" width="11.3984375" style="15"/>
-    <col min="15" max="15" width="11.3984375" style="10"/>
+    <col min="3" max="3" width="34.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" style="2" customWidth="1"/>
+    <col min="9" max="14" width="11.42578125" style="15"/>
+    <col min="15" max="15" width="11.42578125" style="10"/>
     <col min="16" max="16" width="16" customWidth="1"/>
     <col min="17" max="17" width="18" customWidth="1"/>
     <col min="18" max="18" width="12" style="11" customWidth="1"/>
-    <col min="19" max="19" width="11.3984375" style="10"/>
+    <col min="19" max="19" width="11.42578125" style="10"/>
     <col min="21" max="21" width="20" customWidth="1"/>
     <col min="22" max="22" width="14" customWidth="1"/>
     <col min="23" max="23" width="26" customWidth="1"/>
     <col min="24" max="24" width="16" customWidth="1"/>
     <col min="25" max="25" width="12" style="11" customWidth="1"/>
-    <col min="26" max="26" width="29.3984375" style="10" customWidth="1"/>
+    <col min="26" max="26" width="29.42578125" style="10" customWidth="1"/>
     <col min="28" max="28" width="21" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="5" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:29" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -9983,7 +9970,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>7</v>
       </c>
@@ -10080,7 +10067,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>8</v>
       </c>
@@ -10177,7 +10164,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9</v>
       </c>
@@ -10274,7 +10261,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>10</v>
       </c>
@@ -10371,7 +10358,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>11</v>
       </c>
@@ -10468,7 +10455,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>12</v>
       </c>
@@ -10565,7 +10552,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>19</v>
       </c>
@@ -10662,7 +10649,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>20</v>
       </c>
@@ -10759,7 +10746,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>21</v>
       </c>
@@ -10856,7 +10843,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>22</v>
       </c>
@@ -10953,7 +10940,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>23</v>
       </c>
@@ -11050,7 +11037,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>24</v>
       </c>
@@ -11147,7 +11134,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>25</v>
       </c>
@@ -11244,7 +11231,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>26</v>
       </c>
@@ -11341,7 +11328,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>32</v>
       </c>
@@ -11438,7 +11425,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>33</v>
       </c>
@@ -11535,7 +11522,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:31" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>34</v>
       </c>
@@ -11632,7 +11619,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:31" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>35</v>
       </c>
@@ -11730,7 +11717,7 @@
       </c>
       <c r="AE19" s="13"/>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>36</v>
       </c>
@@ -11827,7 +11814,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>44</v>
       </c>
@@ -11924,7 +11911,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>45</v>
       </c>
@@ -12021,7 +12008,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>46</v>
       </c>
@@ -12118,7 +12105,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>47</v>
       </c>
@@ -12215,7 +12202,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>48</v>
       </c>
@@ -12312,7 +12299,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>49</v>
       </c>
@@ -12409,7 +12396,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>50</v>
       </c>
@@ -12506,7 +12493,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>51</v>
       </c>
@@ -12603,7 +12590,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="35">
         <v>0</v>
       </c>
@@ -12700,7 +12687,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="35">
         <v>1</v>
       </c>
@@ -12797,7 +12784,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="35">
         <v>2</v>
       </c>
@@ -12894,7 +12881,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="35">
         <v>3</v>
       </c>
@@ -12991,7 +12978,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="35">
         <v>4</v>
       </c>
@@ -13088,7 +13075,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="35">
         <v>5</v>
       </c>
@@ -13185,7 +13172,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="35">
         <v>6</v>
       </c>
@@ -13282,7 +13269,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="35">
         <v>13</v>
       </c>
@@ -13379,7 +13366,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="35">
         <v>14</v>
       </c>
@@ -13476,7 +13463,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="35">
         <v>15</v>
       </c>
@@ -13573,7 +13560,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="35">
         <v>16</v>
       </c>
@@ -13670,7 +13657,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="35">
         <v>17</v>
       </c>
@@ -13767,7 +13754,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="35">
         <v>18</v>
       </c>
@@ -13864,7 +13851,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="35">
         <v>27</v>
       </c>
@@ -13961,7 +13948,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="43" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="35">
         <v>28</v>
       </c>
@@ -14058,7 +14045,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="44" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="35">
         <v>29</v>
       </c>
@@ -14155,7 +14142,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="35">
         <v>30</v>
       </c>
@@ -14252,7 +14239,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="35">
         <v>31</v>
       </c>
@@ -14349,7 +14336,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="35">
         <v>37</v>
       </c>
@@ -14446,7 +14433,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="48" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="35">
         <v>38</v>
       </c>
@@ -14543,7 +14530,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="49" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="35">
         <v>39</v>
       </c>
@@ -14640,7 +14627,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="50" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="35">
         <v>40</v>
       </c>
@@ -14737,7 +14724,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="51" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="35">
         <v>41</v>
       </c>
@@ -14834,7 +14821,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="52" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="35">
         <v>42</v>
       </c>
@@ -14931,7 +14918,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="53" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:29" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="35">
         <v>43</v>
       </c>

</xml_diff>